<commit_message>
Update teams master spreadsheet
</commit_message>
<xml_diff>
--- a/src/data/teams-master.xlsx
+++ b/src/data/teams-master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\wwfc\wwfc-website\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A23E287-4DC3-4E9D-AE69-120D9A8B40F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E447FE-CB06-4597-A438-604791B3D1AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7DF92C9-0D00-4B55-9052-44BB95C1396F}"/>
   </bookViews>
@@ -50,7 +50,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N7" authorId="0" shapeId="0" xr:uid="{15D9EEE2-CA5C-43BC-8B01-BAD97442DCCA}">
+    <comment ref="N6" authorId="0" shapeId="0" xr:uid="{15D9EEE2-CA5C-43BC-8B01-BAD97442DCCA}">
       <text>
         <r>
           <rPr>
@@ -74,10 +74,10 @@
         </r>
       </text>
     </comment>
-    <comment ref="K12" authorId="0" shapeId="0" xr:uid="{CA909996-4AD5-4A8E-BC32-A84A0EF3DC22}">
+    <comment ref="K11" authorId="0" shapeId="0" xr:uid="{CA909996-4AD5-4A8E-BC32-A84A0EF3DC22}">
       <text/>
     </comment>
-    <comment ref="N12" authorId="0" shapeId="0" xr:uid="{EA1A2A5E-A06B-40B8-AD76-10A0C357D3D9}">
+    <comment ref="N11" authorId="0" shapeId="0" xr:uid="{EA1A2A5E-A06B-40B8-AD76-10A0C357D3D9}">
       <text>
         <r>
           <rPr>
@@ -91,13 +91,13 @@
         </r>
       </text>
     </comment>
-    <comment ref="N13" authorId="0" shapeId="0" xr:uid="{CDFEB8DC-D67E-4B6C-8EDB-0209B7067E46}">
+    <comment ref="N12" authorId="0" shapeId="0" xr:uid="{CDFEB8DC-D67E-4B6C-8EDB-0209B7067E46}">
       <text/>
     </comment>
-    <comment ref="K14" authorId="0" shapeId="0" xr:uid="{42DD0172-6C19-48BB-B243-CCA7486AD89C}">
+    <comment ref="K13" authorId="0" shapeId="0" xr:uid="{42DD0172-6C19-48BB-B243-CCA7486AD89C}">
       <text/>
     </comment>
-    <comment ref="K15" authorId="0" shapeId="0" xr:uid="{70B6D392-BBF5-4F37-A24C-C6D0CB98E777}">
+    <comment ref="K14" authorId="0" shapeId="0" xr:uid="{70B6D392-BBF5-4F37-A24C-C6D0CB98E777}">
       <text>
         <r>
           <rPr>
@@ -121,7 +121,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K17" authorId="0" shapeId="0" xr:uid="{1FD260F4-F1C1-4801-BDA5-7AB52B8FF343}">
+    <comment ref="K16" authorId="0" shapeId="0" xr:uid="{1FD260F4-F1C1-4801-BDA5-7AB52B8FF343}">
       <text>
         <r>
           <rPr>
@@ -145,10 +145,10 @@
         </r>
       </text>
     </comment>
-    <comment ref="K19" authorId="0" shapeId="0" xr:uid="{27ED2F2B-6702-43E5-8352-44F7B654D995}">
+    <comment ref="K18" authorId="0" shapeId="0" xr:uid="{27ED2F2B-6702-43E5-8352-44F7B654D995}">
       <text/>
     </comment>
-    <comment ref="N19" authorId="0" shapeId="0" xr:uid="{E563512F-E421-48EF-A838-552E02BD8306}">
+    <comment ref="N18" authorId="0" shapeId="0" xr:uid="{E563512F-E421-48EF-A838-552E02BD8306}">
       <text>
         <r>
           <rPr>
@@ -162,10 +162,10 @@
         </r>
       </text>
     </comment>
-    <comment ref="N20" authorId="0" shapeId="0" xr:uid="{B0CF4723-74B5-407C-A895-E1C19159F65D}">
+    <comment ref="N19" authorId="0" shapeId="0" xr:uid="{B0CF4723-74B5-407C-A895-E1C19159F65D}">
       <text/>
     </comment>
-    <comment ref="N23" authorId="0" shapeId="0" xr:uid="{FF7BB13A-1F8C-455B-A5E7-FE64CDF23808}">
+    <comment ref="N22" authorId="0" shapeId="0" xr:uid="{FF7BB13A-1F8C-455B-A5E7-FE64CDF23808}">
       <text/>
     </comment>
   </commentList>
@@ -173,7 +173,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="220">
   <si>
     <t>section</t>
   </si>
@@ -861,18 +861,6 @@
       </rPr>
       <t>We're real people who live and breathe property, design, and doing things differently. Independent, unapologetic, and full of fresh perspective, we're a team of visionaries, lettings pros, creatives and developers who see beyond the usual.</t>
     </r>
-  </si>
-  <si>
-    <t>Rebels</t>
-  </si>
-  <si>
-    <t>Jack Morement</t>
-  </si>
-  <si>
-    <t>The Rebels are a newly formed team, starting at u8 and playing 5v5 Footnall</t>
-  </si>
-  <si>
-    <t>rebels@wwfc.org.uk</t>
   </si>
 </sst>
 </file>
@@ -1881,7 +1869,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52D2363D-25C8-4F80-BF49-26CC19A643F2}">
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.77734375" customWidth="1"/>
@@ -2032,38 +2020,40 @@
         <v>163</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>22</v>
       </c>
       <c r="B4">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="C4" t="s">
-        <v>220</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>221</v>
+        <v>29</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>30</v>
       </c>
       <c r="F4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>222</v>
+      <c r="H4" s="3" t="s">
+        <v>122</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="L4" s="9"/>
-      <c r="M4" s="2"/>
-    </row>
-    <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+      <c r="L4" s="10"/>
+      <c r="N4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="28.2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -2071,64 +2061,63 @@
         <v>2017</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="L5" s="10"/>
+      <c r="H5" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I5" t="s">
+        <v>36</v>
+      </c>
       <c r="N5" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" ht="28.2" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="40.200000000000003" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>22</v>
       </c>
       <c r="B6">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
       </c>
-      <c r="H6" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I6" t="s">
-        <v>36</v>
+      <c r="H6" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="N6" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" ht="40.200000000000003" x14ac:dyDescent="0.3">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="55.8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -2136,77 +2125,74 @@
         <v>2016</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>43</v>
+      <c r="H7" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="I7" t="s">
+        <v>46</v>
       </c>
       <c r="N7" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="55.8" x14ac:dyDescent="0.3">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="42" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>22</v>
       </c>
       <c r="B8">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="I8" t="s">
-        <v>46</v>
-      </c>
-      <c r="N8" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="42" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="55.8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
       <c r="B9">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="F9" t="s">
         <v>14</v>
@@ -2215,10 +2201,13 @@
         <v>1</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>125</v>
+        <v>81</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
+      </c>
+      <c r="N9" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="55.8" x14ac:dyDescent="0.3">
@@ -2229,10 +2218,10 @@
         <v>2014</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>35</v>
@@ -2244,16 +2233,28 @@
         <v>1</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
+      </c>
+      <c r="J10" t="s">
+        <v>150</v>
+      </c>
+      <c r="K10" t="s">
+        <v>149</v>
+      </c>
+      <c r="L10" t="s">
+        <v>151</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>152</v>
       </c>
       <c r="N10" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="55.8" x14ac:dyDescent="0.3">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -2261,10 +2262,10 @@
         <v>2014</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D11" t="s">
-        <v>56</v>
+        <v>204</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>35</v>
@@ -2276,28 +2277,28 @@
         <v>1</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>58</v>
+        <v>80</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="J11" t="s">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="K11" t="s">
-        <v>149</v>
-      </c>
-      <c r="L11" t="s">
-        <v>151</v>
+        <v>201</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>202</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>152</v>
+        <v>203</v>
       </c>
       <c r="N11" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -2305,10 +2306,10 @@
         <v>2014</v>
       </c>
       <c r="C12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>204</v>
+        <v>63</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>35</v>
@@ -2319,40 +2320,28 @@
       <c r="G12" t="b">
         <v>1</v>
       </c>
-      <c r="H12" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="J12" t="s">
-        <v>200</v>
-      </c>
-      <c r="K12" t="s">
-        <v>201</v>
-      </c>
-      <c r="L12" s="16" t="s">
-        <v>202</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>203</v>
+      <c r="H12" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>64</v>
       </c>
       <c r="N12" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>22</v>
       </c>
       <c r="B13">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D13" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>35</v>
@@ -2364,16 +2353,25 @@
         <v>1</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
+      </c>
+      <c r="J13" t="s">
+        <v>197</v>
+      </c>
+      <c r="K13" t="s">
+        <v>198</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>199</v>
       </c>
       <c r="N13" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="45" x14ac:dyDescent="0.7">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -2381,13 +2379,13 @@
         <v>2013</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>35</v>
+        <v>26</v>
+      </c>
+      <c r="E14" s="1">
+        <v>19</v>
       </c>
       <c r="F14" t="s">
         <v>14</v>
@@ -2395,84 +2393,84 @@
       <c r="G14" t="b">
         <v>1</v>
       </c>
-      <c r="H14" s="7" t="s">
-        <v>79</v>
+      <c r="H14" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>67</v>
+        <v>27</v>
       </c>
       <c r="J14" t="s">
-        <v>197</v>
+        <v>164</v>
       </c>
       <c r="K14" t="s">
-        <v>198</v>
-      </c>
-      <c r="L14" s="16" t="s">
-        <v>199</v>
+        <v>171</v>
+      </c>
+      <c r="L14" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>166</v>
       </c>
       <c r="N14" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="45" x14ac:dyDescent="0.7">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="B15">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="C15" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="D15" t="s">
-        <v>26</v>
-      </c>
-      <c r="E15" s="1">
-        <v>19</v>
+        <v>69</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="F15" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G15" t="b">
         <v>1</v>
       </c>
-      <c r="H15" s="5" t="s">
-        <v>32</v>
+      <c r="H15" s="7" t="s">
+        <v>78</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="J15" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="K15" t="s">
-        <v>171</v>
-      </c>
-      <c r="L15" s="15" t="s">
-        <v>165</v>
+        <v>148</v>
+      </c>
+      <c r="L15" t="s">
+        <v>146</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="N15" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="134.4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>9</v>
       </c>
       <c r="B16">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="C16" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D16" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="F16" t="s">
         <v>11</v>
@@ -2481,25 +2479,28 @@
         <v>1</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="J16" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="K16" t="s">
-        <v>148</v>
-      </c>
-      <c r="L16" t="s">
-        <v>146</v>
+        <v>141</v>
+      </c>
+      <c r="L16" s="12" t="s">
+        <v>144</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="134.4" x14ac:dyDescent="0.3">
+        <v>142</v>
+      </c>
+      <c r="N16" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -2507,10 +2508,10 @@
         <v>2010</v>
       </c>
       <c r="C17" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D17" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>51</v>
@@ -2522,124 +2523,109 @@
         <v>1</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="J17" t="s">
-        <v>140</v>
+        <v>167</v>
       </c>
       <c r="K17" t="s">
-        <v>141</v>
-      </c>
-      <c r="L17" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>142</v>
+        <v>168</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="M17" t="s">
+        <v>170</v>
       </c>
       <c r="N17" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="64.8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18">
-        <v>2010</v>
+        <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="D18" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="F18" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G18" t="b">
         <v>1</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="J18" t="s">
-        <v>167</v>
+        <v>208</v>
       </c>
       <c r="K18" t="s">
-        <v>168</v>
-      </c>
-      <c r="L18" s="8" t="s">
-        <v>169</v>
+        <v>205</v>
+      </c>
+      <c r="L18" s="19" t="s">
+        <v>219</v>
       </c>
       <c r="M18" t="s">
-        <v>170</v>
+        <v>207</v>
       </c>
       <c r="N18" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="64.8" x14ac:dyDescent="0.3">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>193</v>
       </c>
       <c r="D19" t="s">
         <v>85</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="F19" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G19" t="b">
         <v>1</v>
       </c>
-      <c r="H19" s="7" t="s">
-        <v>87</v>
+      <c r="H19" s="3" t="s">
+        <v>194</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="J19" t="s">
-        <v>208</v>
-      </c>
-      <c r="K19" t="s">
-        <v>205</v>
-      </c>
-      <c r="L19" s="19" t="s">
-        <v>219</v>
-      </c>
-      <c r="M19" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="N19" t="s">
-        <v>182</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>193</v>
+        <v>90</v>
       </c>
       <c r="D20" t="s">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F20" t="s">
         <v>11</v>
@@ -2648,52 +2634,55 @@
         <v>1</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>194</v>
+        <v>92</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="N20" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="27.6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="J20" t="s">
+        <v>192</v>
+      </c>
+      <c r="K20" t="s">
+        <v>191</v>
+      </c>
+      <c r="L20" s="18"/>
+      <c r="M20" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>22</v>
+      </c>
+      <c r="B21">
+        <v>2012</v>
       </c>
       <c r="C21" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D21" t="s">
-        <v>38</v>
+        <v>94</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F21" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="G21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>92</v>
+        <v>211</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J21" t="s">
-        <v>192</v>
-      </c>
-      <c r="K21" t="s">
-        <v>191</v>
-      </c>
-      <c r="L21" s="18"/>
-      <c r="M21" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+        <v>96</v>
+      </c>
+      <c r="L21" s="17" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -2701,31 +2690,37 @@
         <v>2012</v>
       </c>
       <c r="C22" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D22" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>95</v>
       </c>
       <c r="F22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G22" t="b">
-        <v>0</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>211</v>
+        <v>1</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>210</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="L22" s="17" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+      <c r="J22" t="s">
+        <v>97</v>
+      </c>
+      <c r="K22" t="s">
+        <v>172</v>
+      </c>
+      <c r="N22" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -2733,34 +2728,40 @@
         <v>2012</v>
       </c>
       <c r="C23" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D23" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="F23" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G23" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>210</v>
+        <v>0</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>212</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="J23" t="s">
-        <v>97</v>
+        <v>140</v>
       </c>
       <c r="K23" t="s">
-        <v>172</v>
+        <v>141</v>
+      </c>
+      <c r="L23" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="M23" t="s">
+        <v>142</v>
       </c>
       <c r="N23" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
@@ -2768,46 +2769,46 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="C24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D24" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="F24" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="J24" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="K24" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="L24" s="13" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="M24" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="N24" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -2815,40 +2816,29 @@
         <v>2011</v>
       </c>
       <c r="C25" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>106</v>
       </c>
       <c r="F25" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G25" t="b">
         <v>1</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="J25" t="s">
-        <v>154</v>
-      </c>
-      <c r="K25" t="s">
-        <v>153</v>
-      </c>
-      <c r="L25" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="M25" t="s">
-        <v>155</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="L25" s="14"/>
       <c r="N25" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
@@ -2856,16 +2846,16 @@
         <v>22</v>
       </c>
       <c r="B26">
-        <v>2011</v>
+        <v>2010</v>
       </c>
       <c r="C26" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D26" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="F26" t="s">
         <v>14</v>
@@ -2874,125 +2864,95 @@
         <v>1</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="L26" s="14"/>
-      <c r="N26" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:14" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>22</v>
       </c>
       <c r="B27">
-        <v>2010</v>
+        <v>2009</v>
       </c>
       <c r="C27" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D27" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="F27" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G27" t="b">
         <v>1</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L27" s="14"/>
-    </row>
-    <row r="28" spans="1:14" ht="172.8" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+      <c r="L27" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="118.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>22</v>
       </c>
       <c r="B28">
-        <v>2009</v>
+        <v>2007</v>
       </c>
       <c r="C28" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D28" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="F28" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G28" t="b">
         <v>1</v>
       </c>
-      <c r="H28" s="3" t="s">
-        <v>216</v>
+      <c r="H28" s="8" t="s">
+        <v>120</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
+      </c>
+      <c r="J28" t="s">
+        <v>157</v>
+      </c>
+      <c r="K28" t="s">
+        <v>160</v>
       </c>
       <c r="L28" s="13" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" ht="118.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>22</v>
-      </c>
-      <c r="B29">
-        <v>2007</v>
-      </c>
-      <c r="C29" t="s">
-        <v>118</v>
-      </c>
-      <c r="D29" t="s">
-        <v>119</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="F29" t="s">
-        <v>14</v>
-      </c>
-      <c r="G29" t="b">
-        <v>1</v>
-      </c>
-      <c r="H29" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="J29" t="s">
-        <v>157</v>
-      </c>
-      <c r="K29" t="s">
-        <v>160</v>
-      </c>
-      <c r="L29" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="M29" t="s">
+      <c r="M28" t="s">
         <v>158</v>
       </c>
-      <c r="N29" t="s">
+      <c r="N28" t="s">
         <v>183</v>
       </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="E29" s="1"/>
+      <c r="L29" s="14"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E30" s="1"/>
-      <c r="L30" s="14"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E31" s="1"/>
@@ -3120,45 +3080,41 @@
     <row r="72" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E72" s="1"/>
     </row>
-    <row r="73" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E73" s="1"/>
-    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="I15" r:id="rId1" xr:uid="{1DDE6441-190C-4FB5-88D6-BD2305EF1037}"/>
-    <hyperlink ref="I5" r:id="rId2" xr:uid="{464AEA72-DD90-493F-B1EA-F064D72E58ED}"/>
-    <hyperlink ref="I7" r:id="rId3" xr:uid="{C3FB2965-268C-4260-B12A-BF3B3D06E0D2}"/>
-    <hyperlink ref="I9" r:id="rId4" display="mailto:wyfc.rockets@gmail.com" xr:uid="{94AEF066-47C6-4A5E-810B-679E732621D3}"/>
-    <hyperlink ref="I10" r:id="rId5" display="mailto:wyfc.dragons@gmail.com" xr:uid="{1199F452-4FFD-4443-A221-CB874C056106}"/>
-    <hyperlink ref="I11" r:id="rId6" display="mailto:wyfc.lightning@gmail.com" xr:uid="{45D87601-135B-4938-9E30-D9DBAB839D74}"/>
-    <hyperlink ref="I13" r:id="rId7" xr:uid="{F964898C-E695-43AF-ABF1-6B2AEEF41DA5}"/>
-    <hyperlink ref="I14" r:id="rId8" xr:uid="{A277BAD3-7950-4856-83E2-B3B805CDE7FB}"/>
-    <hyperlink ref="I16" r:id="rId9" xr:uid="{4FFCD438-A697-4E2B-862E-AEB7FBA70D2C}"/>
-    <hyperlink ref="I17" r:id="rId10" xr:uid="{ACE97416-41EF-4E1A-9C81-891544793CCB}"/>
-    <hyperlink ref="I18" r:id="rId11" xr:uid="{F740E58B-F83F-407C-8A2A-205A90C20C2B}"/>
-    <hyperlink ref="I19" r:id="rId12" xr:uid="{C1A06EC3-1156-4297-856C-F9D31C5D8517}"/>
-    <hyperlink ref="I20" r:id="rId13" xr:uid="{A83EFAE6-7C65-4944-B61E-D63B500BFEC2}"/>
-    <hyperlink ref="I21" r:id="rId14" xr:uid="{D586C23B-DE62-4E2A-A1BE-6E6679A289EE}"/>
-    <hyperlink ref="I22" r:id="rId15" xr:uid="{0CC4A010-A755-4529-B3BC-88360D529C8F}"/>
-    <hyperlink ref="I23" r:id="rId16" xr:uid="{66D5CA7C-D658-4136-9E90-8186A7EC0D49}"/>
-    <hyperlink ref="I24" r:id="rId17" xr:uid="{EB731D00-8BAD-493A-B65D-D9FDCB99DA24}"/>
-    <hyperlink ref="I25" r:id="rId18" xr:uid="{FB09940C-8366-4603-B0B9-5A7F0FE53856}"/>
-    <hyperlink ref="I26" r:id="rId19" xr:uid="{1F0DF1FE-3341-4D07-9881-D7032C2BCFD6}"/>
-    <hyperlink ref="I27" r:id="rId20" xr:uid="{34FD123B-32E2-4723-A99F-B214EF856113}"/>
-    <hyperlink ref="I28" r:id="rId21" xr:uid="{1DA03B7F-3218-4DA3-89B0-AEB5BF3B2793}"/>
-    <hyperlink ref="I29" r:id="rId22" xr:uid="{9A40DF52-6BA2-4984-9B40-763FAC09DA40}"/>
+    <hyperlink ref="I14" r:id="rId1" xr:uid="{1DDE6441-190C-4FB5-88D6-BD2305EF1037}"/>
+    <hyperlink ref="I4" r:id="rId2" xr:uid="{464AEA72-DD90-493F-B1EA-F064D72E58ED}"/>
+    <hyperlink ref="I6" r:id="rId3" xr:uid="{C3FB2965-268C-4260-B12A-BF3B3D06E0D2}"/>
+    <hyperlink ref="I8" r:id="rId4" display="mailto:wyfc.rockets@gmail.com" xr:uid="{94AEF066-47C6-4A5E-810B-679E732621D3}"/>
+    <hyperlink ref="I9" r:id="rId5" display="mailto:wyfc.dragons@gmail.com" xr:uid="{1199F452-4FFD-4443-A221-CB874C056106}"/>
+    <hyperlink ref="I10" r:id="rId6" display="mailto:wyfc.lightning@gmail.com" xr:uid="{45D87601-135B-4938-9E30-D9DBAB839D74}"/>
+    <hyperlink ref="I12" r:id="rId7" xr:uid="{F964898C-E695-43AF-ABF1-6B2AEEF41DA5}"/>
+    <hyperlink ref="I13" r:id="rId8" xr:uid="{A277BAD3-7950-4856-83E2-B3B805CDE7FB}"/>
+    <hyperlink ref="I15" r:id="rId9" xr:uid="{4FFCD438-A697-4E2B-862E-AEB7FBA70D2C}"/>
+    <hyperlink ref="I16" r:id="rId10" xr:uid="{ACE97416-41EF-4E1A-9C81-891544793CCB}"/>
+    <hyperlink ref="I17" r:id="rId11" xr:uid="{F740E58B-F83F-407C-8A2A-205A90C20C2B}"/>
+    <hyperlink ref="I18" r:id="rId12" xr:uid="{C1A06EC3-1156-4297-856C-F9D31C5D8517}"/>
+    <hyperlink ref="I19" r:id="rId13" xr:uid="{A83EFAE6-7C65-4944-B61E-D63B500BFEC2}"/>
+    <hyperlink ref="I20" r:id="rId14" xr:uid="{D586C23B-DE62-4E2A-A1BE-6E6679A289EE}"/>
+    <hyperlink ref="I21" r:id="rId15" xr:uid="{0CC4A010-A755-4529-B3BC-88360D529C8F}"/>
+    <hyperlink ref="I22" r:id="rId16" xr:uid="{66D5CA7C-D658-4136-9E90-8186A7EC0D49}"/>
+    <hyperlink ref="I23" r:id="rId17" xr:uid="{EB731D00-8BAD-493A-B65D-D9FDCB99DA24}"/>
+    <hyperlink ref="I24" r:id="rId18" xr:uid="{FB09940C-8366-4603-B0B9-5A7F0FE53856}"/>
+    <hyperlink ref="I25" r:id="rId19" xr:uid="{1F0DF1FE-3341-4D07-9881-D7032C2BCFD6}"/>
+    <hyperlink ref="I26" r:id="rId20" xr:uid="{34FD123B-32E2-4723-A99F-B214EF856113}"/>
+    <hyperlink ref="I27" r:id="rId21" xr:uid="{1DA03B7F-3218-4DA3-89B0-AEB5BF3B2793}"/>
+    <hyperlink ref="I28" r:id="rId22" xr:uid="{9A40DF52-6BA2-4984-9B40-763FAC09DA40}"/>
     <hyperlink ref="M3" r:id="rId23" xr:uid="{41620B85-57B4-4EA1-83B0-0EC365818842}"/>
-    <hyperlink ref="M16" r:id="rId24" xr:uid="{334F4A00-D252-43DB-BCCF-7E0762FE4D0A}"/>
-    <hyperlink ref="M11" r:id="rId25" xr:uid="{923F8D44-DFAD-4DE1-8022-AAA409E43920}"/>
-    <hyperlink ref="M17" r:id="rId26" xr:uid="{80BF0B3C-6F43-4D23-98BE-97C5F752891C}"/>
-    <hyperlink ref="M15" r:id="rId27" xr:uid="{9F723FE9-2235-4D80-B338-C2273BDEA705}"/>
-    <hyperlink ref="M21" r:id="rId28" xr:uid="{38A395C6-5484-4F9A-89D4-25C7597D6F80}"/>
-    <hyperlink ref="M12" r:id="rId29" xr:uid="{77B1CEF9-89D1-4450-B781-5912FF963AF3}"/>
-    <hyperlink ref="I4" r:id="rId30" xr:uid="{C04DA833-5EA0-4EC2-B81E-13611A882C0E}"/>
+    <hyperlink ref="M15" r:id="rId24" xr:uid="{334F4A00-D252-43DB-BCCF-7E0762FE4D0A}"/>
+    <hyperlink ref="M10" r:id="rId25" xr:uid="{923F8D44-DFAD-4DE1-8022-AAA409E43920}"/>
+    <hyperlink ref="M16" r:id="rId26" xr:uid="{80BF0B3C-6F43-4D23-98BE-97C5F752891C}"/>
+    <hyperlink ref="M14" r:id="rId27" xr:uid="{9F723FE9-2235-4D80-B338-C2273BDEA705}"/>
+    <hyperlink ref="M20" r:id="rId28" xr:uid="{38A395C6-5484-4F9A-89D4-25C7597D6F80}"/>
+    <hyperlink ref="M11" r:id="rId29" xr:uid="{77B1CEF9-89D1-4450-B781-5912FF963AF3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId31"/>
-  <legacyDrawing r:id="rId32"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId30"/>
+  <legacyDrawing r:id="rId31"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
@@ -3166,7 +3122,7 @@
           <x14:formula1>
             <xm:f>data!$A$1:$A$9</xm:f>
           </x14:formula1>
-          <xm:sqref>F19:F1048576 I8 F1:F17</xm:sqref>
+          <xm:sqref>F18:F1048576 I7 F1:F16</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FA1CACC6-E1C6-4D34-9880-2BA45F8D9BBE}">
           <x14:formula1>

</xml_diff>